<commit_message>
Changed background colour, added singapore call-out box and added Portugal to the database
</commit_message>
<xml_diff>
--- a/data/Program Data.xlsx
+++ b/data/Program Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Documents\GTF-Impact-Map\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s2730428\Documents\GTF-Impact-Map\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC3E499-50CC-4FFF-807E-9C58A6B32A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739ACBF5-638A-404E-AC54-839D33172FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD56EADB-1935-49BD-AB38-7127B858C65A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AD56EADB-1935-49BD-AB38-7127B858C65A}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>Country</t>
   </si>
@@ -262,6 +265,9 @@
   </si>
   <si>
     <t>Ivory Coast</t>
+  </si>
+  <si>
+    <t>Portugal</t>
   </si>
 </sst>
 </file>
@@ -317,10 +323,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}" name="Table1" displayName="Table1" ref="A1:D73" totalsRowShown="0">
-  <autoFilter ref="A1:D73" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D73">
-    <sortCondition ref="A1:A73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}" name="Table1" displayName="Table1" ref="A1:D74" totalsRowShown="0">
+  <autoFilter ref="A1:D74" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D74">
+    <sortCondition ref="A1:A74"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{BB1A4DB9-2749-4819-BDEB-2476FD66E4FC}" name="Country"/>
@@ -333,9 +339,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -373,7 +379,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -479,7 +485,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -621,7 +627,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -629,14 +635,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D6A2811-651E-4A40-8F1F-EACB1DE63CE0}">
-  <dimension ref="A1:D73"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D74"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="34.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="1" max="1" width="34.1796875" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -650,7 +656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -664,7 +670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
@@ -678,7 +684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -692,7 +698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -706,7 +712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -720,7 +726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -734,7 +740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -748,7 +754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -762,7 +768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -776,7 +782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -790,7 +796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -804,7 +810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>63</v>
       </c>
@@ -818,7 +824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -832,7 +838,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -846,7 +852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -860,7 +866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -874,7 +880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>8</v>
       </c>
@@ -888,7 +894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -902,7 +908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>64</v>
       </c>
@@ -916,7 +922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -930,7 +936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>41</v>
       </c>
@@ -944,7 +950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -958,7 +964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -972,7 +978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>65</v>
       </c>
@@ -986,7 +992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1000,7 +1006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -1014,7 +1020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -1028,7 +1034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -1042,7 +1048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>44</v>
       </c>
@@ -1056,7 +1062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>45</v>
       </c>
@@ -1070,7 +1076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>46</v>
       </c>
@@ -1084,7 +1090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>66</v>
       </c>
@@ -1098,7 +1104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1112,7 +1118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>75</v>
       </c>
@@ -1126,7 +1132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -1140,7 +1146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>34</v>
       </c>
@@ -1154,7 +1160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>15</v>
       </c>
@@ -1168,7 +1174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -1182,7 +1188,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>67</v>
       </c>
@@ -1196,7 +1202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>68</v>
       </c>
@@ -1210,7 +1216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>27</v>
       </c>
@@ -1224,7 +1230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>69</v>
       </c>
@@ -1238,7 +1244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>7</v>
       </c>
@@ -1252,7 +1258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>14</v>
       </c>
@@ -1266,7 +1272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -1280,7 +1286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>10</v>
       </c>
@@ -1294,7 +1300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>70</v>
       </c>
@@ -1308,7 +1314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -1322,7 +1328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>47</v>
       </c>
@@ -1336,7 +1342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>17</v>
       </c>
@@ -1350,7 +1356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>71</v>
       </c>
@@ -1364,7 +1370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>48</v>
       </c>
@@ -1378,7 +1384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>49</v>
       </c>
@@ -1392,7 +1398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>19</v>
       </c>
@@ -1406,7 +1412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>9</v>
       </c>
@@ -1420,7 +1426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>50</v>
       </c>
@@ -1434,7 +1440,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>25</v>
       </c>
@@ -1448,7 +1454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>6</v>
       </c>
@@ -1462,199 +1468,213 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
+        <v>76</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>51</v>
       </c>
-      <c r="B60">
-        <v>0</v>
-      </c>
-      <c r="C60">
-        <v>1</v>
-      </c>
-      <c r="D60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+      <c r="B61">
+        <v>0</v>
+      </c>
+      <c r="C61">
+        <v>1</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>52</v>
       </c>
-      <c r="B61">
-        <v>0</v>
-      </c>
-      <c r="C61">
-        <v>1</v>
-      </c>
-      <c r="D61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+      <c r="B62">
+        <v>0</v>
+      </c>
+      <c r="C62">
+        <v>1</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>13</v>
       </c>
-      <c r="B62">
-        <v>1</v>
-      </c>
-      <c r="C62">
-        <v>1</v>
-      </c>
-      <c r="D62">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+      <c r="B63">
+        <v>1</v>
+      </c>
+      <c r="C63">
+        <v>1</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>5</v>
       </c>
-      <c r="B63">
-        <v>1</v>
-      </c>
-      <c r="C63">
-        <v>1</v>
-      </c>
-      <c r="D63">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+      <c r="B64">
+        <v>1</v>
+      </c>
+      <c r="C64">
+        <v>1</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>53</v>
       </c>
-      <c r="B64">
-        <v>0</v>
-      </c>
-      <c r="C64">
-        <v>1</v>
-      </c>
-      <c r="D64">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+      <c r="B65">
+        <v>0</v>
+      </c>
+      <c r="C65">
+        <v>1</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>54</v>
       </c>
-      <c r="B65">
-        <v>0</v>
-      </c>
-      <c r="C65">
-        <v>1</v>
-      </c>
-      <c r="D65">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+      <c r="B66">
+        <v>0</v>
+      </c>
+      <c r="C66">
+        <v>1</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>55</v>
       </c>
-      <c r="B66">
-        <v>0</v>
-      </c>
-      <c r="C66">
-        <v>1</v>
-      </c>
-      <c r="D66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+      <c r="B67">
+        <v>0</v>
+      </c>
+      <c r="C67">
+        <v>1</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>56</v>
       </c>
-      <c r="B67">
-        <v>0</v>
-      </c>
-      <c r="C67">
-        <v>1</v>
-      </c>
-      <c r="D67">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+      <c r="B68">
+        <v>0</v>
+      </c>
+      <c r="C68">
+        <v>1</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>57</v>
       </c>
-      <c r="B68">
-        <v>0</v>
-      </c>
-      <c r="C68">
-        <v>1</v>
-      </c>
-      <c r="D68">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+      <c r="B69">
+        <v>0</v>
+      </c>
+      <c r="C69">
+        <v>1</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>72</v>
       </c>
-      <c r="B69">
-        <v>0</v>
-      </c>
-      <c r="C69">
-        <v>0</v>
-      </c>
-      <c r="D69">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+      <c r="B70">
+        <v>0</v>
+      </c>
+      <c r="C70">
+        <v>0</v>
+      </c>
+      <c r="D70">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>73</v>
       </c>
-      <c r="B70">
-        <v>0</v>
-      </c>
-      <c r="C70">
-        <v>0</v>
-      </c>
-      <c r="D70">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+      <c r="B71">
+        <v>0</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>59</v>
       </c>
-      <c r="B71">
-        <v>0</v>
-      </c>
-      <c r="C71">
-        <v>1</v>
-      </c>
-      <c r="D71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="B72">
+        <v>0</v>
+      </c>
+      <c r="C72">
+        <v>1</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>35</v>
       </c>
-      <c r="B72">
-        <v>1</v>
-      </c>
-      <c r="C72">
-        <v>1</v>
-      </c>
-      <c r="D72">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="B73">
+        <v>1</v>
+      </c>
+      <c r="C73">
+        <v>1</v>
+      </c>
+      <c r="D73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>74</v>
       </c>
-      <c r="B73">
-        <v>0</v>
-      </c>
-      <c r="C73">
-        <v>0</v>
-      </c>
-      <c r="D73">
+      <c r="B74">
+        <v>0</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+      <c r="D74">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Database and disclaimer update
</commit_message>
<xml_diff>
--- a/data/Program Data.xlsx
+++ b/data/Program Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Documents\Global Talent Fund\GTF-Impact-Map\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78E1933B-FF9C-420A-97E9-C9ED3A24C2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB83E6A-F119-47F7-8EFF-E4F7C49C4DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AD56EADB-1935-49BD-AB38-7127B858C65A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>Country</t>
   </si>
@@ -265,6 +265,12 @@
   </si>
   <si>
     <t>Türkiye, Republic of</t>
+  </si>
+  <si>
+    <t>Egypt</t>
+  </si>
+  <si>
+    <t>Peru</t>
   </si>
 </sst>
 </file>
@@ -320,8 +326,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}" name="Table1" displayName="Table1" ref="A1:D74" totalsRowShown="0">
-  <autoFilter ref="A1:D74" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}" name="Table1" displayName="Table1" ref="A1:D76" totalsRowShown="0">
+  <autoFilter ref="A1:D76" xr:uid="{7EBCA682-35F6-443E-9599-16C39EBD80EE}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:D74">
     <sortCondition ref="A1:A74"/>
   </sortState>
@@ -632,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D6A2811-651E-4A40-8F1F-EACB1DE63CE0}">
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.140625" customWidth="1"/>
@@ -1673,6 +1679,34 @@
       </c>
       <c r="D74">
         <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75">
+        <v>0</v>
+      </c>
+      <c r="C75">
+        <v>1</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76">
+        <v>0</v>
+      </c>
+      <c r="C76">
+        <v>1</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>